<commit_message>
Incluídas as perdas de projeto e excedente
</commit_message>
<xml_diff>
--- a/appOrcam/static/arquivos/Preco_m2 esfiha e kibe Onda E (version 1).xlsx
+++ b/appOrcam/static/arquivos/Preco_m2 esfiha e kibe Onda E (version 1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Documents\GitHub\Dj_srcx_Orcamento\appOrcam\static\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{AF721066-096F-430E-84A5-B00074874F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{84A79ADB-0EF6-401E-8379-A426B6C19800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{67754E85-EF51-4CB9-B61E-3CED47B47D87}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="55">
   <si>
     <t>id</t>
   </si>
@@ -216,6 +216,12 @@
   </si>
   <si>
     <t>Custos Unitários de materiais</t>
+  </si>
+  <si>
+    <t>área total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">área aparas </t>
   </si>
 </sst>
 </file>
@@ -245,10 +251,10 @@
     <numFmt numFmtId="182" formatCode="&quot;R$&quot;\ #,##0.000\ &quot;por chapa&quot;"/>
     <numFmt numFmtId="184" formatCode="&quot;R$&quot;\ #,##0.000\ &quot;seladora&quot;"/>
     <numFmt numFmtId="185" formatCode="&quot;R$&quot;\ #,##0.000"/>
-    <numFmt numFmtId="186" formatCode="#,##0\ &quot;unidades&quot;"/>
     <numFmt numFmtId="187" formatCode="&quot;Csuto de fabricação: &quot;\ &quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="188" formatCode="&quot;Capac_nominal: &quot;#,##0\ &quot;unidades&quot;"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -427,8 +433,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -644,6 +657,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="35">
     <border>
@@ -1102,7 +1127,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1336,7 +1361,6 @@
     <xf numFmtId="167" fontId="21" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="186" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="180" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="43" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1369,11 +1393,13 @@
     <xf numFmtId="187" fontId="16" fillId="38" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="185" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="179" fontId="24" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="171" fontId="20" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="185" fontId="20" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="185" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="20" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1680,15 +1706,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>670112</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>133351</xdr:rowOff>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>110941</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>727263</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>98333</xdr:rowOff>
+      <xdr:colOff>704851</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>87129</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -1703,13 +1729,13 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm rot="16200000" flipH="1" flipV="1">
-          <a:off x="643359" y="3443428"/>
+          <a:off x="620947" y="3230518"/>
           <a:ext cx="3943070" cy="2679327"/>
         </a:xfrm>
         <a:prstGeom prst="bentConnector4">
           <a:avLst>
             <a:gd name="adj1" fmla="val -5804"/>
-            <a:gd name="adj2" fmla="val 108541"/>
+            <a:gd name="adj2" fmla="val 121506"/>
           </a:avLst>
         </a:prstGeom>
         <a:ln>
@@ -3619,19 +3645,22 @@
     <col min="9" max="9" width="30.140625" customWidth="1"/>
     <col min="10" max="10" width="24.140625" customWidth="1"/>
     <col min="11" max="11" width="26.42578125" customWidth="1"/>
-    <col min="12" max="12" width="39" customWidth="1"/>
+    <col min="12" max="12" width="45.85546875" customWidth="1"/>
     <col min="13" max="13" width="47.140625" customWidth="1"/>
     <col min="14" max="14" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="M2" s="96"/>
-      <c r="N2" s="97" t="s">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="M2" s="95"/>
+      <c r="N2" s="96" t="s">
         <v>47</v>
       </c>
-      <c r="O2" s="96"/>
-      <c r="P2" s="96"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -3649,22 +3678,25 @@
       <c r="F3" t="s">
         <v>4</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>38</v>
+      </c>
       <c r="I3" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" s="97" t="s">
+        <v>54</v>
+      </c>
+      <c r="M3" s="96" t="s">
         <v>46</v>
       </c>
-      <c r="N3" s="97" t="s">
+      <c r="N3" s="96" t="s">
         <v>49</v>
       </c>
-      <c r="O3" s="97" t="s">
+      <c r="O3" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="97" t="s">
+      <c r="P3" s="96" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3684,14 +3716,14 @@
       <c r="F4" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="1">
+      <c r="H4" s="1">
         <v>1</v>
       </c>
-      <c r="J4" s="1">
-        <f>+P4-I4/100*D4/100-I4/100*E4/100</f>
-        <v>0.23449999999999999</v>
-      </c>
-      <c r="K4" s="96" t="s">
+      <c r="J4" s="3">
+        <f>((D4-2*$G$2)*(E4-2*$G$2))/10000</f>
+        <v>0.22439999999999999</v>
+      </c>
+      <c r="K4" s="95" t="s">
         <v>6</v>
       </c>
       <c r="L4" t="s">
@@ -3704,7 +3736,7 @@
         <v>1000</v>
       </c>
       <c r="O4" s="1">
-        <v>2.92</v>
+        <v>1.78</v>
       </c>
       <c r="P4" s="3">
         <f>+D4/100*E4/100</f>
@@ -3727,14 +3759,14 @@
       <c r="F5" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="1">
+      <c r="H5" s="1">
         <v>1</v>
       </c>
-      <c r="J5" s="1">
-        <f>+P5-0.01*D5/100-0.01*E5/100</f>
-        <v>0.308</v>
-      </c>
-      <c r="K5" s="96" t="s">
+      <c r="J5" s="3">
+        <f t="shared" ref="J5:J8" si="0">((D5-2*$G$2)*(E5-2*$G$2))/10000</f>
+        <v>0.2964</v>
+      </c>
+      <c r="K5" s="95" t="s">
         <v>8</v>
       </c>
       <c r="L5" t="s">
@@ -3747,7 +3779,7 @@
         <v>600</v>
       </c>
       <c r="O5" s="1">
-        <v>2.92</v>
+        <v>1.78</v>
       </c>
       <c r="P5" s="3">
         <f>+D5/100*E5/100</f>
@@ -3770,14 +3802,14 @@
       <c r="F6" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="1">
+      <c r="H6" s="1">
         <v>1</v>
       </c>
-      <c r="J6" s="1">
-        <f>+P6-0.01*D6/100-0.01*E6/100</f>
-        <v>0.39150000000000001</v>
-      </c>
-      <c r="K6" s="96" t="s">
+      <c r="J6" s="3">
+        <f t="shared" si="0"/>
+        <v>0.37840000000000001</v>
+      </c>
+      <c r="K6" s="95" t="s">
         <v>9</v>
       </c>
       <c r="L6" t="s">
@@ -3790,7 +3822,7 @@
         <v>600</v>
       </c>
       <c r="O6" s="1">
-        <v>2.92</v>
+        <v>1.78</v>
       </c>
       <c r="P6" s="3">
         <f>+D6/100*E6/100</f>
@@ -3813,14 +3845,14 @@
       <c r="F7" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="1">
+      <c r="H7" s="1">
         <v>1</v>
       </c>
-      <c r="J7" s="1">
-        <f>+P7-0.01*D7/100-0.01*E7/100</f>
-        <v>0.48499999999999999</v>
-      </c>
-      <c r="K7" s="96" t="s">
+      <c r="J7" s="3">
+        <f t="shared" si="0"/>
+        <v>0.47039999999999998</v>
+      </c>
+      <c r="K7" s="95" t="s">
         <v>10</v>
       </c>
       <c r="L7" t="s">
@@ -3833,7 +3865,7 @@
         <v>2500</v>
       </c>
       <c r="O7" s="1">
-        <v>2.92</v>
+        <v>1.78</v>
       </c>
       <c r="P7" s="3">
         <f>+D7/100*E7/100</f>
@@ -3856,14 +3888,14 @@
       <c r="F8" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="1">
+      <c r="H8" s="1">
         <v>1</v>
       </c>
-      <c r="J8" s="1">
-        <f>+P8-0.01*D8/100-0.01*E8/100</f>
-        <v>0.58850000000000013</v>
-      </c>
-      <c r="K8" s="96" t="s">
+      <c r="J8" s="3">
+        <f t="shared" si="0"/>
+        <v>0.57240000000000002</v>
+      </c>
+      <c r="K8" s="95" t="s">
         <v>11</v>
       </c>
       <c r="L8" t="s">
@@ -3876,7 +3908,7 @@
         <v>5000</v>
       </c>
       <c r="O8" s="1">
-        <v>2.92</v>
+        <v>1.78</v>
       </c>
       <c r="P8" s="3">
         <f>+D8/100*E8/100</f>
@@ -3919,10 +3951,10 @@
       <c r="D13" s="23"/>
     </row>
     <row r="14" spans="2:16" ht="21" x14ac:dyDescent="0.35">
-      <c r="C14" s="94" t="s">
+      <c r="C14" s="93" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="102" t="s">
+      <c r="D14" s="101" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3943,20 +3975,20 @@
     <row r="17" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C17" s="32">
         <f>+(VLOOKUP(C6,$K$4:$P$8,6,0)/$C$11)*VLOOKUP(C14,$L$4:$P$8,4,0)*IF(C11&gt;1,2,1)</f>
-        <v>1.1826000000000001</v>
+        <v>0.7209000000000001</v>
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="20"/>
       <c r="H17" s="32">
         <f>+C17</f>
-        <v>1.1826000000000001</v>
+        <v>0.7209000000000001</v>
       </c>
       <c r="I17" s="33"/>
       <c r="J17" s="20"/>
-      <c r="L17" s="95">
+      <c r="L17" s="94">
         <v>600</v>
       </c>
-      <c r="M17" s="95"/>
+      <c r="M17" s="94"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C18" s="24"/>
@@ -3982,24 +4014,29 @@
       <c r="H20" s="24"/>
       <c r="I20" s="25"/>
     </row>
-    <row r="21" spans="3:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C21" s="34">
         <f>SUM(C17:D19)</f>
-        <v>1.3826000000000001</v>
+        <v>0.92090000000000005</v>
       </c>
       <c r="D21" s="35"/>
       <c r="H21" s="34">
         <f>SUM(H17:I19)</f>
-        <v>1.3826000000000001</v>
+        <v>0.92090000000000005</v>
       </c>
       <c r="I21" s="35"/>
       <c r="L21" s="107">
         <f>+H21</f>
-        <v>1.3826000000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="3:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="3:13" x14ac:dyDescent="0.25">
+        <v>0.92090000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="L22" s="108"/>
+    </row>
+    <row r="23" spans="3:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L23" s="108"/>
+    </row>
+    <row r="24" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C24" s="84" t="str">
         <f>CONCATENATE("Custos de impressão + Corte para ",$C$28," 
 capac_nominal: ",VLOOKUP($C$28,$L$4:$N$9,3,0)," chapa/hora
@@ -4022,11 +4059,12 @@
       <c r="I24" s="82"/>
       <c r="J24" s="82"/>
       <c r="K24" s="85"/>
+      <c r="L24" s="108"/>
       <c r="M24" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="3:13" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:13" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C25" s="86"/>
       <c r="D25" s="83"/>
       <c r="E25" s="83"/>
@@ -4035,6 +4073,7 @@
       <c r="I25" s="83"/>
       <c r="J25" s="83"/>
       <c r="K25" s="87"/>
+      <c r="L25" s="108"/>
     </row>
     <row r="26" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C26" s="36" t="s">
@@ -4049,23 +4088,25 @@
       <c r="I26" s="37"/>
       <c r="J26" s="37"/>
       <c r="K26" s="38"/>
+      <c r="L26" s="108"/>
       <c r="M26" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="3:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C27" s="39"/>
       <c r="E27" s="40"/>
       <c r="F27" s="41"/>
       <c r="H27" s="39"/>
       <c r="J27" s="40"/>
       <c r="K27" s="41"/>
-      <c r="M27" s="89">
+      <c r="L27" s="108"/>
+      <c r="M27" s="105">
         <v>600</v>
       </c>
     </row>
-    <row r="28" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="C28" s="104" t="str">
+    <row r="28" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="C28" s="103" t="str">
         <f>+C14</f>
         <v>Wonder 2</v>
       </c>
@@ -4097,15 +4138,15 @@
         <f>+$J$28/H12</f>
         <v>1.034</v>
       </c>
-      <c r="L28" s="108">
+      <c r="L28" s="109">
         <f>+K28*M27/M28</f>
-        <v>0.62039999999999995</v>
+        <v>1.034</v>
       </c>
       <c r="M28" s="18">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="29" spans="3:13" x14ac:dyDescent="0.25">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="29" spans="3:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C29" s="66"/>
       <c r="D29" s="40"/>
       <c r="E29" s="40"/>
@@ -4114,12 +4155,13 @@
       <c r="I29" s="40"/>
       <c r="J29" s="40"/>
       <c r="K29" s="41"/>
-      <c r="M29" s="89">
+      <c r="L29" s="108"/>
+      <c r="M29" s="105">
         <v>2500</v>
       </c>
     </row>
-    <row r="30" spans="3:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C30" s="103" t="str">
+    <row r="30" spans="3:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C30" s="102" t="str">
         <f>IF(D14&lt;&gt;"",D14,"")</f>
         <v>Century</v>
       </c>
@@ -4151,15 +4193,16 @@
         <f>+J30/$H$12*IF($H$12&gt;1,2,1)</f>
         <v>7.0800000000000002E-2</v>
       </c>
-      <c r="L30" s="108">
+      <c r="L30" s="109">
         <f>+(K30*M29/M30)</f>
-        <v>0.17699999999999999</v>
+        <v>0.29499999999999998</v>
       </c>
       <c r="M30" s="18">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="31" spans="3:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <f>+M28</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="31" spans="3:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C31" s="49">
         <f>SUM(F28:F30)</f>
         <v>1.1048</v>
@@ -4174,10 +4217,11 @@
       <c r="I31" s="50"/>
       <c r="J31" s="47"/>
       <c r="K31" s="48"/>
-      <c r="L31" s="109"/>
-    </row>
-    <row r="32" spans="3:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="M32" s="92"/>
+      <c r="L31" s="110"/>
+    </row>
+    <row r="32" spans="3:13" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L32" s="108"/>
+      <c r="M32" s="91"/>
     </row>
     <row r="33" spans="3:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C33" s="36" t="s">
@@ -4192,8 +4236,9 @@
       <c r="I33" s="37"/>
       <c r="J33" s="37"/>
       <c r="K33" s="38"/>
-    </row>
-    <row r="34" spans="3:16" x14ac:dyDescent="0.25">
+      <c r="L33" s="108"/>
+    </row>
+    <row r="34" spans="3:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C34" s="39"/>
       <c r="D34" s="40"/>
       <c r="E34" s="40"/>
@@ -4202,11 +4247,12 @@
       <c r="I34" s="40"/>
       <c r="J34" s="40"/>
       <c r="K34" s="41"/>
-      <c r="M34" s="89">
+      <c r="L34" s="108"/>
+      <c r="M34" s="105">
         <v>5000</v>
       </c>
     </row>
-    <row r="35" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C35" s="67" t="str">
         <f>+L8</f>
         <v>Seladora</v>
@@ -4239,22 +4285,23 @@
         <f>+J35*VLOOKUP(H35,$L$4:$M$9,2,0)</f>
         <v>7.0799999999999995E-3</v>
       </c>
-      <c r="L35" s="108">
+      <c r="L35" s="109">
         <f>+(K35*M34/M35)</f>
-        <v>3.5400000000000001E-2</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="M35" s="18">
-        <v>1000</v>
+        <f>+M30</f>
+        <v>600</v>
       </c>
     </row>
     <row r="36" spans="3:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C36" s="98">
+      <c r="C36" s="97">
         <f>SUM(F35)</f>
         <v>7.0799999999999995E-3</v>
       </c>
-      <c r="D36" s="99"/>
-      <c r="E36" s="99"/>
-      <c r="F36" s="100"/>
+      <c r="D36" s="98"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="99"/>
       <c r="H36" s="68">
         <f>SUM(K35)</f>
         <v>7.0799999999999995E-3</v>
@@ -4262,27 +4309,27 @@
       <c r="I36" s="69"/>
       <c r="J36" s="69"/>
       <c r="K36" s="70"/>
-      <c r="M36" s="93"/>
+      <c r="M36" s="92"/>
     </row>
     <row r="37" spans="3:16" x14ac:dyDescent="0.25">
-      <c r="C37" s="101">
+      <c r="C37" s="100">
         <f>+C36+C31</f>
         <v>1.11188</v>
       </c>
-      <c r="D37" s="101"/>
-      <c r="E37" s="101"/>
-      <c r="F37" s="101"/>
-      <c r="H37" s="101">
+      <c r="D37" s="100"/>
+      <c r="E37" s="100"/>
+      <c r="F37" s="100"/>
+      <c r="H37" s="100">
         <f>+H36+H31</f>
         <v>1.11188</v>
       </c>
-      <c r="I37" s="101"/>
-      <c r="J37" s="101"/>
-      <c r="K37" s="101"/>
-      <c r="L37" s="105"/>
-      <c r="M37" s="105"/>
-      <c r="N37" s="105"/>
-      <c r="O37" s="105"/>
+      <c r="I37" s="100"/>
+      <c r="J37" s="100"/>
+      <c r="K37" s="100"/>
+      <c r="L37" s="104"/>
+      <c r="M37" s="104"/>
+      <c r="N37" s="104"/>
+      <c r="O37" s="104"/>
     </row>
     <row r="38" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="39" spans="3:16" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4308,28 +4355,28 @@
       </c>
     </row>
     <row r="40" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="3:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C41" s="55">
         <f>+C21+C31+C36+C39</f>
-        <v>2.7944800000000001</v>
+        <v>2.3327800000000001</v>
       </c>
       <c r="D41" s="56"/>
       <c r="E41" s="56"/>
       <c r="F41" s="57"/>
       <c r="H41" s="55">
         <f>+H21+H31+H36+H39</f>
-        <v>2.7944800000000001</v>
+        <v>2.3327800000000001</v>
       </c>
       <c r="I41" s="56"/>
       <c r="J41" s="56"/>
       <c r="K41" s="57"/>
-      <c r="L41" s="110">
+      <c r="L41" s="111">
         <f>SUM(L28:L30,L35,L39+L21)</f>
-        <v>2.5154000000000001</v>
+        <v>2.6089000000000002</v>
       </c>
       <c r="M41" s="55">
         <f>+H21+M30+M36+M39</f>
-        <v>1001.6826</v>
+        <v>601.22089999999992</v>
       </c>
       <c r="N41" s="56"/>
       <c r="O41" s="56"/>
@@ -4349,7 +4396,7 @@
       <c r="I43" s="59"/>
       <c r="J43" s="59"/>
       <c r="K43" s="60"/>
-      <c r="M43" s="90">
+      <c r="M43" s="89">
         <f>+H43</f>
         <v>0.1</v>
       </c>
@@ -4406,32 +4453,32 @@
     <row r="48" spans="3:16" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C48" s="61">
         <f>+C41/(1-C43)</f>
-        <v>3.1049777777777776</v>
+        <v>2.5919777777777777</v>
       </c>
       <c r="D48" s="62"/>
       <c r="E48" s="62"/>
       <c r="F48" s="63"/>
       <c r="H48" s="61">
         <f>+H41/(1-H43)</f>
-        <v>3.1049777777777776</v>
+        <v>2.5919777777777777</v>
       </c>
       <c r="I48" s="62"/>
       <c r="J48" s="62"/>
       <c r="K48" s="63"/>
       <c r="L48" s="106">
         <f>+L41*(1+H43)</f>
-        <v>2.7669400000000004</v>
+        <v>2.8697900000000005</v>
       </c>
       <c r="M48" s="61">
         <f>+M41/(1-M43)</f>
-        <v>1112.9806666666666</v>
+        <v>668.0232222222221</v>
       </c>
       <c r="N48" s="62"/>
       <c r="O48" s="62"/>
       <c r="P48" s="63"/>
     </row>
     <row r="49" spans="12:12" x14ac:dyDescent="0.25">
-      <c r="L49" s="91"/>
+      <c r="L49" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="37">

</xml_diff>